<commit_message>
Designed additional elements for RoB part
</commit_message>
<xml_diff>
--- a/Datasets/primary_info.xlsx
+++ b/Datasets/primary_info.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniofleicester-my.sharepoint.com/personal/crn4_leicester_ac_uk/Documents/PhD/WP2/3. Create tool/Datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="420" documentId="13_ncr:1_{009773F8-B678-42EB-90F1-9F0C232CDCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{907FD90A-E196-465D-9806-713BC011015B}"/>
+  <xr:revisionPtr revIDLastSave="428" documentId="13_ncr:1_{009773F8-B678-42EB-90F1-9F0C232CDCBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7AC4BA5-6815-43AA-ABB9-2837077CCF59}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{E19E56DC-86BE-4713-A769-C66B74D62B61}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{E19E56DC-86BE-4713-A769-C66B74D62B61}"/>
   </bookViews>
   <sheets>
     <sheet name="Studies" sheetId="1" r:id="rId1"/>
     <sheet name="GRADE" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Studies!$A$1:$X$178</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1146,7 +1149,7 @@
         <v>44317</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
         <v>36</v>
@@ -1158,10 +1161,10 @@
         <v>31</v>
       </c>
       <c r="G5">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H5">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="I5" t="s">
         <v>31</v>
@@ -1170,22 +1173,10 @@
         <v>31</v>
       </c>
       <c r="K5">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>229</v>
-      </c>
-      <c r="M5">
-        <v>1.527301</v>
-      </c>
-      <c r="N5">
-        <v>1.0687709999999999</v>
-      </c>
-      <c r="O5">
-        <v>0.68051099999999998</v>
-      </c>
-      <c r="P5">
-        <v>1.67855</v>
+        <v>224</v>
       </c>
       <c r="X5" t="s">
         <v>58</v>
@@ -1199,7 +1190,7 @@
         <v>44317</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
         <v>37</v>
@@ -1211,7 +1202,7 @@
         <v>31</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6">
         <v>20</v>
@@ -1223,22 +1214,10 @@
         <v>31</v>
       </c>
       <c r="K6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L6">
         <v>20</v>
-      </c>
-      <c r="M6">
-        <v>5.8058999999999999E-2</v>
-      </c>
-      <c r="N6">
-        <v>0.5</v>
-      </c>
-      <c r="O6">
-        <v>4.9182999999999998E-2</v>
-      </c>
-      <c r="P6">
-        <v>5.0830599999999997</v>
       </c>
       <c r="X6" t="s">
         <v>58</v>
@@ -1252,10 +1231,10 @@
         <v>44317</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
         <v>31</v>
@@ -1264,10 +1243,10 @@
         <v>31</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="H7">
-        <v>179</v>
+        <v>228</v>
       </c>
       <c r="I7" t="s">
         <v>31</v>
@@ -1276,22 +1255,22 @@
         <v>31</v>
       </c>
       <c r="K7">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="L7">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="M7">
-        <v>0.40039599999999997</v>
+        <v>88.5</v>
       </c>
       <c r="N7">
-        <v>0.47765400000000002</v>
+        <v>0.877193</v>
       </c>
       <c r="O7">
-        <v>0.197579</v>
+        <v>0.54556800000000005</v>
       </c>
       <c r="P7">
-        <v>1.154744</v>
+        <v>1.4103969999999999</v>
       </c>
       <c r="X7" t="s">
         <v>22</v>
@@ -1302,13 +1281,13 @@
         <v>35</v>
       </c>
       <c r="B8" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
         <v>31</v>
@@ -1317,10 +1296,10 @@
         <v>31</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="I8" t="s">
         <v>31</v>
@@ -1329,25 +1308,25 @@
         <v>31</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L8">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="M8">
-        <v>0.115594</v>
+        <v>11.5</v>
       </c>
       <c r="N8">
-        <v>0.54901999999999995</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="O8">
-        <v>0.10613400000000001</v>
+        <v>0.3</v>
       </c>
       <c r="P8">
-        <v>2.8400099999999999</v>
+        <v>4.22</v>
       </c>
       <c r="X8" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.35">
@@ -1358,10 +1337,10 @@
         <v>44958</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -1370,10 +1349,10 @@
         <v>31</v>
       </c>
       <c r="G9">
-        <v>10</v>
+        <v>171</v>
       </c>
       <c r="H9">
-        <v>69</v>
+        <v>228</v>
       </c>
       <c r="I9" t="s">
         <v>31</v>
@@ -1382,22 +1361,22 @@
         <v>31</v>
       </c>
       <c r="K9">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="L9">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="M9">
-        <v>0.415265</v>
+        <v>3.500273</v>
       </c>
       <c r="N9">
-        <v>1.213768</v>
+        <v>0.984375</v>
       </c>
       <c r="O9">
-        <v>0.51014700000000002</v>
+        <v>0.86388100000000001</v>
       </c>
       <c r="P9">
-        <v>2.8878629999999998</v>
+        <v>1.1216759999999999</v>
       </c>
       <c r="X9" t="s">
         <v>22</v>
@@ -1411,10 +1390,10 @@
         <v>44958</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
         <v>31</v>
@@ -1423,10 +1402,10 @@
         <v>31</v>
       </c>
       <c r="G10">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="H10">
-        <v>257</v>
+        <v>51</v>
       </c>
       <c r="I10" t="s">
         <v>31</v>
@@ -1435,25 +1414,25 @@
         <v>31</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="L10">
-        <v>254</v>
+        <v>50</v>
       </c>
       <c r="M10">
-        <v>6.8178000000000002E-2</v>
+        <v>0.28551799999999999</v>
       </c>
       <c r="N10">
-        <v>4.9416339999999996</v>
+        <v>1.4161220000000001</v>
       </c>
       <c r="O10">
-        <v>0.58139600000000002</v>
+        <v>0.89650200000000002</v>
       </c>
       <c r="P10">
-        <v>42.001891000000001</v>
+        <v>2.2369180000000002</v>
       </c>
       <c r="X10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
@@ -1464,10 +1443,10 @@
         <v>44958</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
         <v>31</v>
@@ -1476,10 +1455,10 @@
         <v>31</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>257</v>
       </c>
       <c r="H11">
-        <v>231</v>
+        <v>320</v>
       </c>
       <c r="I11" t="s">
         <v>31</v>
@@ -1488,22 +1467,22 @@
         <v>31</v>
       </c>
       <c r="K11">
-        <v>19</v>
+        <v>130</v>
       </c>
       <c r="L11">
-        <v>240</v>
+        <v>163</v>
       </c>
       <c r="M11">
-        <v>0.70235199999999998</v>
+        <v>6.6862830000000004</v>
       </c>
       <c r="N11">
-        <v>0.76554999999999995</v>
+        <v>1.0069950000000001</v>
       </c>
       <c r="O11">
-        <v>0.39319599999999999</v>
+        <v>0.91621699999999995</v>
       </c>
       <c r="P11">
-        <v>1.4905200000000001</v>
+        <v>1.106768</v>
       </c>
       <c r="X11" t="s">
         <v>22</v>
@@ -1514,26 +1493,26 @@
         <v>35</v>
       </c>
       <c r="B12" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12">
+        <v>31</v>
+      </c>
+      <c r="H12">
         <v>43</v>
       </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G12">
-        <v>25</v>
-      </c>
-      <c r="H12">
-        <v>228</v>
-      </c>
       <c r="I12" t="s">
         <v>31</v>
       </c>
@@ -1541,25 +1520,25 @@
         <v>31</v>
       </c>
       <c r="K12">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="L12">
-        <v>105</v>
+        <v>43</v>
       </c>
       <c r="M12">
-        <v>0.74170499999999995</v>
+        <v>0.72387299999999999</v>
       </c>
       <c r="N12">
-        <v>0.95943000000000001</v>
+        <v>1.107143</v>
       </c>
       <c r="O12">
-        <v>0.50169799999999998</v>
+        <v>0.83082</v>
       </c>
       <c r="P12">
-        <v>1.834781</v>
+        <v>1.475368</v>
       </c>
       <c r="X12" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.35">
@@ -1570,10 +1549,10 @@
         <v>44958</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
         <v>31</v>
@@ -1582,10 +1561,10 @@
         <v>31</v>
       </c>
       <c r="G13">
-        <v>2</v>
+        <v>3832</v>
       </c>
       <c r="H13">
-        <v>40</v>
+        <v>5795</v>
       </c>
       <c r="I13" t="s">
         <v>31</v>
@@ -1594,25 +1573,25 @@
         <v>31</v>
       </c>
       <c r="K13">
-        <v>10</v>
+        <v>3822</v>
       </c>
       <c r="L13">
-        <v>39</v>
+        <v>5763</v>
       </c>
       <c r="M13">
-        <v>0.147929</v>
+        <v>88.006018999999995</v>
       </c>
       <c r="N13">
-        <v>0.19500000000000001</v>
+        <v>0.99707999999999997</v>
       </c>
       <c r="O13">
-        <v>4.5617999999999999E-2</v>
+        <v>0.97145099999999995</v>
       </c>
       <c r="P13">
-        <v>0.83355599999999996</v>
+        <v>1.023385</v>
       </c>
       <c r="X13" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.35">
@@ -1623,10 +1602,10 @@
         <v>44958</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
         <v>31</v>
@@ -1635,10 +1614,10 @@
         <v>31</v>
       </c>
       <c r="G14">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="H14">
-        <v>36</v>
+        <v>80</v>
       </c>
       <c r="I14" t="s">
         <v>31</v>
@@ -1647,25 +1626,25 @@
         <v>31</v>
       </c>
       <c r="K14">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="L14">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="M14">
-        <v>0.58537700000000004</v>
+        <v>0.79803299999999999</v>
       </c>
       <c r="N14">
-        <v>0.87654299999999996</v>
+        <v>0.95652199999999998</v>
       </c>
       <c r="O14">
-        <v>0.42244700000000002</v>
+        <v>0.72766799999999998</v>
       </c>
       <c r="P14">
-        <v>1.818754</v>
+        <v>1.25735</v>
       </c>
       <c r="X14" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.35">
@@ -1673,13 +1652,13 @@
         <v>35</v>
       </c>
       <c r="B15" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="E15" t="s">
         <v>31</v>
@@ -1688,10 +1667,10 @@
         <v>31</v>
       </c>
       <c r="G15">
-        <v>352</v>
+        <v>34</v>
       </c>
       <c r="H15">
-        <v>1074</v>
+        <v>235</v>
       </c>
       <c r="I15" t="s">
         <v>31</v>
@@ -1700,25 +1679,25 @@
         <v>31</v>
       </c>
       <c r="K15">
-        <v>300</v>
+        <v>31</v>
       </c>
       <c r="L15">
-        <v>904</v>
+        <v>229</v>
       </c>
       <c r="M15">
-        <v>18.837778</v>
+        <v>1.527301</v>
       </c>
       <c r="N15">
-        <v>0.98760999999999999</v>
+        <v>1.0687709999999999</v>
       </c>
       <c r="O15">
-        <v>0.87063699999999999</v>
+        <v>0.68051099999999998</v>
       </c>
       <c r="P15">
-        <v>1.1202989999999999</v>
+        <v>1.67855</v>
       </c>
       <c r="X15" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.35">
@@ -1732,7 +1711,7 @@
         <v>95</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
         <v>31</v>
@@ -1741,10 +1720,10 @@
         <v>31</v>
       </c>
       <c r="G16">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="I16" t="s">
         <v>31</v>
@@ -1753,25 +1732,25 @@
         <v>31</v>
       </c>
       <c r="K16">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L16">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="M16">
-        <v>0.48129300000000003</v>
+        <v>5.8058999999999999E-2</v>
       </c>
       <c r="N16">
-        <v>0.65359500000000004</v>
+        <v>0.5</v>
       </c>
       <c r="O16">
-        <v>0.29219099999999998</v>
+        <v>4.9182999999999998E-2</v>
       </c>
       <c r="P16">
-        <v>1.462008</v>
+        <v>5.0830599999999997</v>
       </c>
       <c r="X16" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.35">
@@ -1779,13 +1758,13 @@
         <v>35</v>
       </c>
       <c r="B17" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D17" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E17" t="s">
         <v>31</v>
@@ -1794,10 +1773,10 @@
         <v>31</v>
       </c>
       <c r="G17">
-        <v>141</v>
+        <v>7</v>
       </c>
       <c r="H17">
-        <v>614</v>
+        <v>179</v>
       </c>
       <c r="I17" t="s">
         <v>31</v>
@@ -1806,22 +1785,22 @@
         <v>31</v>
       </c>
       <c r="K17">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="L17">
-        <v>307</v>
+        <v>171</v>
       </c>
       <c r="M17">
-        <v>4.4525050000000004</v>
+        <v>0.40039599999999997</v>
       </c>
       <c r="N17">
-        <v>1.119048</v>
+        <v>0.47765400000000002</v>
       </c>
       <c r="O17">
-        <v>0.85979899999999998</v>
+        <v>0.197579</v>
       </c>
       <c r="P17">
-        <v>1.456466</v>
+        <v>1.154744</v>
       </c>
       <c r="X17" t="s">
         <v>22</v>
@@ -1832,13 +1811,13 @@
         <v>35</v>
       </c>
       <c r="B18" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D18" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E18" t="s">
         <v>31</v>
@@ -1847,10 +1826,10 @@
         <v>31</v>
       </c>
       <c r="G18">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H18">
-        <v>320</v>
+        <v>228</v>
       </c>
       <c r="I18" t="s">
         <v>31</v>
@@ -1859,22 +1838,22 @@
         <v>31</v>
       </c>
       <c r="K18">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L18">
-        <v>163</v>
+        <v>105</v>
       </c>
       <c r="M18">
-        <v>0.83953800000000001</v>
+        <v>0.74170499999999995</v>
       </c>
       <c r="N18">
-        <v>1.055134</v>
+        <v>0.95943000000000001</v>
       </c>
       <c r="O18">
-        <v>0.57369300000000001</v>
+        <v>0.50169799999999998</v>
       </c>
       <c r="P18">
-        <v>1.9406000000000001</v>
+        <v>1.834781</v>
       </c>
       <c r="X18" t="s">
         <v>22</v>
@@ -1885,52 +1864,52 @@
         <v>35</v>
       </c>
       <c r="B19" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19">
+        <v>8</v>
+      </c>
+      <c r="H19">
+        <v>51</v>
+      </c>
+      <c r="I19" t="s">
+        <v>31</v>
+      </c>
+      <c r="J19" t="s">
+        <v>31</v>
+      </c>
+      <c r="K19">
+        <v>12</v>
+      </c>
+      <c r="L19">
         <v>50</v>
       </c>
-      <c r="E19" t="s">
-        <v>31</v>
-      </c>
-      <c r="F19" t="s">
-        <v>31</v>
-      </c>
-      <c r="G19">
-        <v>6</v>
-      </c>
-      <c r="H19">
-        <v>43</v>
-      </c>
-      <c r="I19" t="s">
-        <v>31</v>
-      </c>
-      <c r="J19" t="s">
-        <v>31</v>
-      </c>
-      <c r="K19">
-        <v>11</v>
-      </c>
-      <c r="L19">
-        <v>43</v>
-      </c>
       <c r="M19">
-        <v>0.38482899999999998</v>
+        <v>0.48129300000000003</v>
       </c>
       <c r="N19">
-        <v>0.54545500000000002</v>
+        <v>0.65359500000000004</v>
       </c>
       <c r="O19">
-        <v>0.221667</v>
+        <v>0.29219099999999998</v>
       </c>
       <c r="P19">
-        <v>1.3421940000000001</v>
+        <v>1.462008</v>
       </c>
       <c r="X19" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.35">
@@ -1991,13 +1970,13 @@
         <v>35</v>
       </c>
       <c r="B21" s="1">
-        <v>44958</v>
+        <v>44317</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E21" t="s">
         <v>31</v>
@@ -2006,10 +1985,10 @@
         <v>31</v>
       </c>
       <c r="G21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H21">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="I21" t="s">
         <v>31</v>
@@ -2021,22 +2000,22 @@
         <v>14</v>
       </c>
       <c r="L21">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="M21">
-        <v>0.51285800000000004</v>
+        <v>0.66848399999999997</v>
       </c>
       <c r="N21">
-        <v>0.56064700000000001</v>
+        <v>0.71428599999999998</v>
       </c>
       <c r="O21">
-        <v>0.25703399999999998</v>
+        <v>0.360792</v>
       </c>
       <c r="P21">
-        <v>1.222893</v>
+        <v>1.4141220000000001</v>
       </c>
       <c r="X21" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.35">
@@ -2050,7 +2029,7 @@
         <v>95</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="E22" t="s">
         <v>31</v>
@@ -2059,10 +2038,10 @@
         <v>31</v>
       </c>
       <c r="G22">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>462</v>
+        <v>17</v>
       </c>
       <c r="I22" t="s">
         <v>31</v>
@@ -2071,25 +2050,25 @@
         <v>31</v>
       </c>
       <c r="K22">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="L22">
-        <v>462</v>
+        <v>14</v>
       </c>
       <c r="M22">
-        <v>3.0239199999999999</v>
+        <v>0.115594</v>
       </c>
       <c r="N22">
-        <v>0.830986</v>
+        <v>0.54901999999999995</v>
       </c>
       <c r="O22">
-        <v>0.60324500000000003</v>
+        <v>0.10613400000000001</v>
       </c>
       <c r="P22">
-        <v>1.1447039999999999</v>
+        <v>2.8400099999999999</v>
       </c>
       <c r="X22" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:24" x14ac:dyDescent="0.35">
@@ -2097,13 +2076,13 @@
         <v>35</v>
       </c>
       <c r="B23" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>95</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="E23" t="s">
         <v>31</v>
@@ -2115,7 +2094,7 @@
         <v>10</v>
       </c>
       <c r="H23">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="I23" t="s">
         <v>31</v>
@@ -2124,25 +2103,25 @@
         <v>31</v>
       </c>
       <c r="K23">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="L23">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="M23">
-        <v>0.66848399999999997</v>
+        <v>0.415265</v>
       </c>
       <c r="N23">
-        <v>0.71428599999999998</v>
+        <v>1.213768</v>
       </c>
       <c r="O23">
-        <v>0.360792</v>
+        <v>0.51014700000000002</v>
       </c>
       <c r="P23">
-        <v>1.4141220000000001</v>
+        <v>2.8878629999999998</v>
       </c>
       <c r="X23" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:24" x14ac:dyDescent="0.35">
@@ -2156,7 +2135,7 @@
         <v>95</v>
       </c>
       <c r="D24" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E24" t="s">
         <v>31</v>
@@ -2165,10 +2144,10 @@
         <v>31</v>
       </c>
       <c r="G24">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H24">
-        <v>80</v>
+        <v>257</v>
       </c>
       <c r="I24" t="s">
         <v>31</v>
@@ -2177,25 +2156,25 @@
         <v>31</v>
       </c>
       <c r="K24">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="L24">
-        <v>80</v>
+        <v>254</v>
       </c>
       <c r="M24">
-        <v>0.755104</v>
+        <v>6.8178000000000002E-2</v>
       </c>
       <c r="N24">
-        <v>1.3846149999999999</v>
+        <v>4.9416339999999996</v>
       </c>
       <c r="O24">
-        <v>0.72823499999999997</v>
+        <v>0.58139600000000002</v>
       </c>
       <c r="P24">
-        <v>2.6326100000000001</v>
+        <v>42.001891000000001</v>
       </c>
       <c r="X24" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:24" x14ac:dyDescent="0.35">
@@ -2209,7 +2188,7 @@
         <v>95</v>
       </c>
       <c r="D25" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E25" t="s">
         <v>31</v>
@@ -2218,10 +2197,10 @@
         <v>31</v>
       </c>
       <c r="G25">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H25">
-        <v>52</v>
+        <v>231</v>
       </c>
       <c r="I25" t="s">
         <v>31</v>
@@ -2230,22 +2209,22 @@
         <v>31</v>
       </c>
       <c r="K25">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="L25">
-        <v>51</v>
+        <v>240</v>
       </c>
       <c r="M25">
-        <v>0.62933399999999995</v>
+        <v>0.70235199999999998</v>
       </c>
       <c r="N25">
-        <v>0.82988200000000001</v>
+        <v>0.76554999999999995</v>
       </c>
       <c r="O25">
-        <v>0.41048899999999999</v>
+        <v>0.39319599999999999</v>
       </c>
       <c r="P25">
-        <v>1.677764</v>
+        <v>1.4905200000000001</v>
       </c>
       <c r="X25" t="s">
         <v>22</v>
@@ -4367,10 +4346,10 @@
         <v>44958</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D60" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="E60" t="s">
         <v>31</v>
@@ -4379,10 +4358,10 @@
         <v>31</v>
       </c>
       <c r="G60">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="H60">
-        <v>235</v>
+        <v>40</v>
       </c>
       <c r="I60" t="s">
         <v>31</v>
@@ -4391,25 +4370,25 @@
         <v>31</v>
       </c>
       <c r="K60">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="L60">
-        <v>229</v>
+        <v>39</v>
       </c>
       <c r="M60">
-        <v>3.0132330000000001</v>
+        <v>0.147929</v>
       </c>
       <c r="N60">
-        <v>1.045771</v>
+        <v>0.19500000000000001</v>
       </c>
       <c r="O60">
-        <v>0.71191599999999999</v>
+        <v>4.5617999999999999E-2</v>
       </c>
       <c r="P60">
-        <v>1.5361880000000001</v>
+        <v>0.83355599999999996</v>
       </c>
       <c r="X60" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:24" x14ac:dyDescent="0.35">
@@ -4420,10 +4399,10 @@
         <v>44958</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D61" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E61" t="s">
         <v>31</v>
@@ -4435,7 +4414,7 @@
         <v>8</v>
       </c>
       <c r="H61">
-        <v>257</v>
+        <v>36</v>
       </c>
       <c r="I61" t="s">
         <v>31</v>
@@ -4444,22 +4423,22 @@
         <v>31</v>
       </c>
       <c r="K61">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="L61">
-        <v>254</v>
+        <v>71</v>
       </c>
       <c r="M61">
-        <v>0.26425199999999999</v>
+        <v>0.58537700000000004</v>
       </c>
       <c r="N61">
-        <v>2.6355379999999999</v>
+        <v>0.87654299999999996</v>
       </c>
       <c r="O61">
-        <v>0.70720499999999997</v>
+        <v>0.42244700000000002</v>
       </c>
       <c r="P61">
-        <v>9.821847</v>
+        <v>1.818754</v>
       </c>
       <c r="X61" t="s">
         <v>58</v>
@@ -4473,10 +4452,10 @@
         <v>44958</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D62" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E62" t="s">
         <v>31</v>
@@ -4485,10 +4464,10 @@
         <v>31</v>
       </c>
       <c r="G62">
-        <v>44</v>
+        <v>352</v>
       </c>
       <c r="H62">
-        <v>228</v>
+        <v>1074</v>
       </c>
       <c r="I62" t="s">
         <v>31</v>
@@ -4497,22 +4476,22 @@
         <v>31</v>
       </c>
       <c r="K62">
-        <v>22</v>
+        <v>300</v>
       </c>
       <c r="L62">
-        <v>105</v>
+        <v>904</v>
       </c>
       <c r="M62">
-        <v>2.154855</v>
+        <v>18.837778</v>
       </c>
       <c r="N62">
-        <v>0.92105300000000001</v>
+        <v>0.98760999999999999</v>
       </c>
       <c r="O62">
-        <v>0.583426</v>
+        <v>0.87063699999999999</v>
       </c>
       <c r="P62">
-        <v>1.454064</v>
+        <v>1.1202989999999999</v>
       </c>
       <c r="X62" t="s">
         <v>22</v>
@@ -4526,10 +4505,10 @@
         <v>44958</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D63" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E63" t="s">
         <v>31</v>
@@ -4538,10 +4517,10 @@
         <v>31</v>
       </c>
       <c r="G63">
-        <v>347</v>
+        <v>141</v>
       </c>
       <c r="H63">
-        <v>701</v>
+        <v>614</v>
       </c>
       <c r="I63" t="s">
         <v>31</v>
@@ -4550,25 +4529,25 @@
         <v>31</v>
       </c>
       <c r="K63">
-        <v>275</v>
+        <v>63</v>
       </c>
       <c r="L63">
-        <v>606</v>
+        <v>307</v>
       </c>
       <c r="M63">
-        <v>26.219619999999999</v>
+        <v>4.4525050000000004</v>
       </c>
       <c r="N63">
-        <v>1.090816</v>
+        <v>1.119048</v>
       </c>
       <c r="O63">
-        <v>0.97233599999999998</v>
+        <v>0.85979899999999998</v>
       </c>
       <c r="P63">
-        <v>1.223733</v>
+        <v>1.456466</v>
       </c>
       <c r="X63" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="64" spans="1:24" x14ac:dyDescent="0.35">
@@ -4579,10 +4558,10 @@
         <v>44958</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D64" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E64" t="s">
         <v>31</v>
@@ -4591,10 +4570,10 @@
         <v>31</v>
       </c>
       <c r="G64">
-        <v>199</v>
+        <v>29</v>
       </c>
       <c r="H64">
-        <v>614</v>
+        <v>320</v>
       </c>
       <c r="I64" t="s">
         <v>31</v>
@@ -4603,22 +4582,22 @@
         <v>31</v>
       </c>
       <c r="K64">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="L64">
-        <v>307</v>
+        <v>163</v>
       </c>
       <c r="M64">
-        <v>9.2676479999999994</v>
+        <v>0.83953800000000001</v>
       </c>
       <c r="N64">
-        <v>1.1569769999999999</v>
+        <v>1.055134</v>
       </c>
       <c r="O64">
-        <v>0.93538299999999996</v>
+        <v>0.57369300000000001</v>
       </c>
       <c r="P64">
-        <v>1.4310659999999999</v>
+        <v>1.9406000000000001</v>
       </c>
       <c r="X64" t="s">
         <v>22</v>
@@ -4632,10 +4611,10 @@
         <v>44958</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D65" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E65" t="s">
         <v>31</v>
@@ -4644,10 +4623,10 @@
         <v>31</v>
       </c>
       <c r="G65">
-        <v>1568</v>
+        <v>6</v>
       </c>
       <c r="H65">
-        <v>5493</v>
+        <v>43</v>
       </c>
       <c r="I65" t="s">
         <v>31</v>
@@ -4656,25 +4635,25 @@
         <v>31</v>
       </c>
       <c r="K65">
-        <v>1568</v>
+        <v>11</v>
       </c>
       <c r="L65">
-        <v>5448</v>
+        <v>43</v>
       </c>
       <c r="M65">
-        <v>59.080393000000001</v>
+        <v>0.38482899999999998</v>
       </c>
       <c r="N65">
-        <v>0.99180800000000002</v>
+        <v>0.54545500000000002</v>
       </c>
       <c r="O65">
-        <v>0.93486999999999998</v>
+        <v>0.221667</v>
       </c>
       <c r="P65">
-        <v>1.0522130000000001</v>
+        <v>1.3421940000000001</v>
       </c>
       <c r="X65" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
     </row>
     <row r="66" spans="1:24" x14ac:dyDescent="0.35">
@@ -4685,10 +4664,10 @@
         <v>44958</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D66" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="E66" t="s">
         <v>31</v>
@@ -4697,10 +4676,10 @@
         <v>31</v>
       </c>
       <c r="G66">
-        <v>171</v>
+        <v>8</v>
       </c>
       <c r="H66">
-        <v>228</v>
+        <v>53</v>
       </c>
       <c r="I66" t="s">
         <v>31</v>
@@ -4709,22 +4688,22 @@
         <v>31</v>
       </c>
       <c r="K66">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="L66">
-        <v>105</v>
+        <v>52</v>
       </c>
       <c r="M66">
-        <v>3.500273</v>
+        <v>0.51285800000000004</v>
       </c>
       <c r="N66">
-        <v>0.984375</v>
+        <v>0.56064700000000001</v>
       </c>
       <c r="O66">
-        <v>0.86388100000000001</v>
+        <v>0.25703399999999998</v>
       </c>
       <c r="P66">
-        <v>1.1216759999999999</v>
+        <v>1.222893</v>
       </c>
       <c r="X66" t="s">
         <v>22</v>
@@ -4738,10 +4717,10 @@
         <v>44958</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D67" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E67" t="s">
         <v>31</v>
@@ -4750,10 +4729,10 @@
         <v>31</v>
       </c>
       <c r="G67">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="H67">
-        <v>51</v>
+        <v>462</v>
       </c>
       <c r="I67" t="s">
         <v>31</v>
@@ -4762,22 +4741,22 @@
         <v>31</v>
       </c>
       <c r="K67">
-        <v>18</v>
+        <v>71</v>
       </c>
       <c r="L67">
-        <v>50</v>
+        <v>462</v>
       </c>
       <c r="M67">
-        <v>0.28551799999999999</v>
+        <v>3.0239199999999999</v>
       </c>
       <c r="N67">
-        <v>1.4161220000000001</v>
+        <v>0.830986</v>
       </c>
       <c r="O67">
-        <v>0.89650200000000002</v>
+        <v>0.60324500000000003</v>
       </c>
       <c r="P67">
-        <v>2.2369180000000002</v>
+        <v>1.1447039999999999</v>
       </c>
       <c r="X67" t="s">
         <v>22</v>
@@ -4791,10 +4770,10 @@
         <v>44958</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D68" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E68" t="s">
         <v>31</v>
@@ -4803,10 +4782,10 @@
         <v>31</v>
       </c>
       <c r="G68">
-        <v>257</v>
+        <v>18</v>
       </c>
       <c r="H68">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="I68" t="s">
         <v>31</v>
@@ -4815,22 +4794,22 @@
         <v>31</v>
       </c>
       <c r="K68">
-        <v>130</v>
+        <v>13</v>
       </c>
       <c r="L68">
-        <v>163</v>
+        <v>80</v>
       </c>
       <c r="M68">
-        <v>6.6862830000000004</v>
+        <v>0.755104</v>
       </c>
       <c r="N68">
-        <v>1.0069950000000001</v>
+        <v>1.3846149999999999</v>
       </c>
       <c r="O68">
-        <v>0.91621699999999995</v>
+        <v>0.72823499999999997</v>
       </c>
       <c r="P68">
-        <v>1.106768</v>
+        <v>2.6326100000000001</v>
       </c>
       <c r="X68" t="s">
         <v>22</v>
@@ -4844,10 +4823,10 @@
         <v>44958</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D69" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E69" t="s">
         <v>31</v>
@@ -4856,10 +4835,10 @@
         <v>31</v>
       </c>
       <c r="G69">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="H69">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="I69" t="s">
         <v>31</v>
@@ -4868,25 +4847,25 @@
         <v>31</v>
       </c>
       <c r="K69">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="L69">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="M69">
-        <v>0.72387299999999999</v>
+        <v>0.62933399999999995</v>
       </c>
       <c r="N69">
-        <v>1.107143</v>
+        <v>0.82988200000000001</v>
       </c>
       <c r="O69">
-        <v>0.83082</v>
+        <v>0.41048899999999999</v>
       </c>
       <c r="P69">
-        <v>1.475368</v>
+        <v>1.677764</v>
       </c>
       <c r="X69" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="70" spans="1:24" x14ac:dyDescent="0.35">
@@ -4897,10 +4876,10 @@
         <v>44958</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D70" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="E70" t="s">
         <v>31</v>
@@ -4909,10 +4888,10 @@
         <v>31</v>
       </c>
       <c r="G70">
-        <v>3832</v>
+        <v>54</v>
       </c>
       <c r="H70">
-        <v>5795</v>
+        <v>228</v>
       </c>
       <c r="I70" t="s">
         <v>31</v>
@@ -4921,22 +4900,22 @@
         <v>31</v>
       </c>
       <c r="K70">
-        <v>3822</v>
+        <v>19</v>
       </c>
       <c r="L70">
-        <v>5763</v>
+        <v>105</v>
       </c>
       <c r="M70">
-        <v>88.006018999999995</v>
+        <v>14.914524999999999</v>
       </c>
       <c r="N70">
-        <v>0.99707999999999997</v>
+        <v>1.308864</v>
       </c>
       <c r="O70">
-        <v>0.97145099999999995</v>
+        <v>0.81892699999999996</v>
       </c>
       <c r="P70">
-        <v>1.023385</v>
+        <v>2.0919159999999999</v>
       </c>
       <c r="X70" t="s">
         <v>22</v>
@@ -4950,10 +4929,10 @@
         <v>44958</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D71" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="E71" t="s">
         <v>31</v>
@@ -4962,10 +4941,10 @@
         <v>31</v>
       </c>
       <c r="G71">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="H71">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="I71" t="s">
         <v>31</v>
@@ -4974,25 +4953,25 @@
         <v>31</v>
       </c>
       <c r="K71">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="L71">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="M71">
-        <v>0.79803299999999999</v>
+        <v>10.218532</v>
       </c>
       <c r="N71">
-        <v>0.95652199999999998</v>
+        <v>0.78</v>
       </c>
       <c r="O71">
-        <v>0.72766799999999998</v>
+        <v>0.42051899999999998</v>
       </c>
       <c r="P71">
-        <v>1.25735</v>
+        <v>1.446785</v>
       </c>
       <c r="X71" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="72" spans="1:24" x14ac:dyDescent="0.35">
@@ -5000,13 +4979,13 @@
         <v>35</v>
       </c>
       <c r="B72" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D72" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E72" t="s">
         <v>31</v>
@@ -5015,10 +4994,10 @@
         <v>31</v>
       </c>
       <c r="G72">
-        <v>0</v>
+        <v>205</v>
       </c>
       <c r="H72">
-        <v>227</v>
+        <v>614</v>
       </c>
       <c r="I72" t="s">
         <v>31</v>
@@ -5027,13 +5006,25 @@
         <v>31</v>
       </c>
       <c r="K72">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="L72">
-        <v>224</v>
+        <v>307</v>
+      </c>
+      <c r="M72">
+        <v>29.240273999999999</v>
+      </c>
+      <c r="N72">
+        <v>1.2654319999999999</v>
+      </c>
+      <c r="O72">
+        <v>1.017868</v>
+      </c>
+      <c r="P72">
+        <v>1.5732090000000001</v>
       </c>
       <c r="X72" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="73" spans="1:24" x14ac:dyDescent="0.35">
@@ -5041,13 +5032,13 @@
         <v>35</v>
       </c>
       <c r="B73" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D73" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E73" t="s">
         <v>31</v>
@@ -5056,10 +5047,10 @@
         <v>31</v>
       </c>
       <c r="G73">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="H73">
-        <v>20</v>
+        <v>320</v>
       </c>
       <c r="I73" t="s">
         <v>31</v>
@@ -5068,10 +5059,22 @@
         <v>31</v>
       </c>
       <c r="K73">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="L73">
-        <v>20</v>
+        <v>163</v>
+      </c>
+      <c r="M73">
+        <v>19.607727000000001</v>
+      </c>
+      <c r="N73">
+        <v>0.98878699999999997</v>
+      </c>
+      <c r="O73">
+        <v>0.68417799999999995</v>
+      </c>
+      <c r="P73">
+        <v>1.429014</v>
       </c>
       <c r="X73" t="s">
         <v>58</v>
@@ -5082,13 +5085,13 @@
         <v>35</v>
       </c>
       <c r="B74" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D74" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E74" t="s">
         <v>31</v>
@@ -5097,10 +5100,10 @@
         <v>31</v>
       </c>
       <c r="G74">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="H74">
-        <v>228</v>
+        <v>1075</v>
       </c>
       <c r="I74" t="s">
         <v>31</v>
@@ -5109,25 +5112,25 @@
         <v>31</v>
       </c>
       <c r="K74">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="L74">
-        <v>105</v>
+        <v>905</v>
       </c>
       <c r="M74">
-        <v>88.5</v>
+        <v>9.301444</v>
       </c>
       <c r="N74">
-        <v>0.877193</v>
+        <v>2.244961</v>
       </c>
       <c r="O74">
-        <v>0.54556800000000005</v>
+        <v>1.163178</v>
       </c>
       <c r="P74">
-        <v>1.4103969999999999</v>
+        <v>4.3328290000000003</v>
       </c>
       <c r="X74" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:24" x14ac:dyDescent="0.35">
@@ -5135,13 +5138,13 @@
         <v>35</v>
       </c>
       <c r="B75" s="1">
-        <v>44317</v>
+        <v>44958</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D75" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E75" t="s">
         <v>31</v>
@@ -5150,10 +5153,10 @@
         <v>31</v>
       </c>
       <c r="G75">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="H75">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="I75" t="s">
         <v>31</v>
@@ -5162,25 +5165,25 @@
         <v>31</v>
       </c>
       <c r="K75">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="L75">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="M75">
-        <v>11.5</v>
+        <v>16.717497999999999</v>
       </c>
       <c r="N75">
-        <v>1.1299999999999999</v>
+        <v>0.86339600000000005</v>
       </c>
       <c r="O75">
-        <v>0.3</v>
+        <v>0.563608</v>
       </c>
       <c r="P75">
-        <v>4.22</v>
+        <v>1.322646</v>
       </c>
       <c r="X75" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="76" spans="1:24" x14ac:dyDescent="0.35">
@@ -5191,10 +5194,10 @@
         <v>44958</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D76" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E76" t="s">
         <v>31</v>
@@ -5203,10 +5206,10 @@
         <v>31</v>
       </c>
       <c r="G76">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="H76">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="I76" t="s">
         <v>31</v>
@@ -5215,25 +5218,25 @@
         <v>31</v>
       </c>
       <c r="K76">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="L76">
-        <v>105</v>
+        <v>229</v>
       </c>
       <c r="M76">
-        <v>14.914524999999999</v>
+        <v>3.0132330000000001</v>
       </c>
       <c r="N76">
-        <v>1.308864</v>
+        <v>1.045771</v>
       </c>
       <c r="O76">
-        <v>0.81892699999999996</v>
+        <v>0.71191599999999999</v>
       </c>
       <c r="P76">
-        <v>2.0919159999999999</v>
+        <v>1.5361880000000001</v>
       </c>
       <c r="X76" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:24" x14ac:dyDescent="0.35">
@@ -5244,10 +5247,10 @@
         <v>44958</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D77" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E77" t="s">
         <v>31</v>
@@ -5256,10 +5259,10 @@
         <v>31</v>
       </c>
       <c r="G77">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H77">
-        <v>40</v>
+        <v>257</v>
       </c>
       <c r="I77" t="s">
         <v>31</v>
@@ -5268,25 +5271,25 @@
         <v>31</v>
       </c>
       <c r="K77">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L77">
-        <v>39</v>
+        <v>254</v>
       </c>
       <c r="M77">
-        <v>10.218532</v>
+        <v>0.26425199999999999</v>
       </c>
       <c r="N77">
-        <v>0.78</v>
+        <v>2.6355379999999999</v>
       </c>
       <c r="O77">
-        <v>0.42051899999999998</v>
+        <v>0.70720499999999997</v>
       </c>
       <c r="P77">
-        <v>1.446785</v>
+        <v>9.821847</v>
       </c>
       <c r="X77" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
     </row>
     <row r="78" spans="1:24" x14ac:dyDescent="0.35">
@@ -5297,10 +5300,10 @@
         <v>44958</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D78" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E78" t="s">
         <v>31</v>
@@ -5309,10 +5312,10 @@
         <v>31</v>
       </c>
       <c r="G78">
-        <v>205</v>
+        <v>44</v>
       </c>
       <c r="H78">
-        <v>614</v>
+        <v>228</v>
       </c>
       <c r="I78" t="s">
         <v>31</v>
@@ -5321,25 +5324,25 @@
         <v>31</v>
       </c>
       <c r="K78">
-        <v>81</v>
+        <v>22</v>
       </c>
       <c r="L78">
-        <v>307</v>
+        <v>105</v>
       </c>
       <c r="M78">
-        <v>29.240273999999999</v>
+        <v>2.154855</v>
       </c>
       <c r="N78">
-        <v>1.2654319999999999</v>
+        <v>0.92105300000000001</v>
       </c>
       <c r="O78">
-        <v>1.017868</v>
+        <v>0.583426</v>
       </c>
       <c r="P78">
-        <v>1.5732090000000001</v>
+        <v>1.454064</v>
       </c>
       <c r="X78" t="s">
-        <v>59</v>
+        <v>22</v>
       </c>
     </row>
     <row r="79" spans="1:24" x14ac:dyDescent="0.35">
@@ -5350,10 +5353,10 @@
         <v>44958</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D79" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E79" t="s">
         <v>31</v>
@@ -5362,10 +5365,10 @@
         <v>31</v>
       </c>
       <c r="G79">
-        <v>66</v>
+        <v>347</v>
       </c>
       <c r="H79">
-        <v>320</v>
+        <v>701</v>
       </c>
       <c r="I79" t="s">
         <v>31</v>
@@ -5374,25 +5377,25 @@
         <v>31</v>
       </c>
       <c r="K79">
-        <v>34</v>
+        <v>275</v>
       </c>
       <c r="L79">
-        <v>163</v>
+        <v>606</v>
       </c>
       <c r="M79">
-        <v>19.607727000000001</v>
+        <v>26.219619999999999</v>
       </c>
       <c r="N79">
-        <v>0.98878699999999997</v>
+        <v>1.090816</v>
       </c>
       <c r="O79">
-        <v>0.68417799999999995</v>
+        <v>0.97233599999999998</v>
       </c>
       <c r="P79">
-        <v>1.429014</v>
+        <v>1.223733</v>
       </c>
       <c r="X79" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="80" spans="1:24" x14ac:dyDescent="0.35">
@@ -5403,10 +5406,10 @@
         <v>44958</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D80" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E80" t="s">
         <v>31</v>
@@ -5415,10 +5418,10 @@
         <v>31</v>
       </c>
       <c r="G80">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="H80">
-        <v>1075</v>
+        <v>614</v>
       </c>
       <c r="I80" t="s">
         <v>31</v>
@@ -5427,25 +5430,25 @@
         <v>31</v>
       </c>
       <c r="K80">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="L80">
-        <v>905</v>
+        <v>307</v>
       </c>
       <c r="M80">
-        <v>9.301444</v>
+        <v>9.2676479999999994</v>
       </c>
       <c r="N80">
-        <v>2.244961</v>
+        <v>1.1569769999999999</v>
       </c>
       <c r="O80">
-        <v>1.163178</v>
+        <v>0.93538299999999996</v>
       </c>
       <c r="P80">
-        <v>4.3328290000000003</v>
+        <v>1.4310659999999999</v>
       </c>
       <c r="X80" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="81" spans="1:24" x14ac:dyDescent="0.35">
@@ -5456,10 +5459,10 @@
         <v>44958</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D81" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E81" t="s">
         <v>31</v>
@@ -5468,10 +5471,10 @@
         <v>31</v>
       </c>
       <c r="G81">
-        <v>22</v>
+        <v>1568</v>
       </c>
       <c r="H81">
-        <v>53</v>
+        <v>5493</v>
       </c>
       <c r="I81" t="s">
         <v>31</v>
@@ -5480,25 +5483,25 @@
         <v>31</v>
       </c>
       <c r="K81">
-        <v>25</v>
+        <v>1568</v>
       </c>
       <c r="L81">
-        <v>52</v>
+        <v>5448</v>
       </c>
       <c r="M81">
-        <v>16.717497999999999</v>
+        <v>59.080393000000001</v>
       </c>
       <c r="N81">
-        <v>0.86339600000000005</v>
+        <v>0.99180800000000002</v>
       </c>
       <c r="O81">
-        <v>0.563608</v>
+        <v>0.93486999999999998</v>
       </c>
       <c r="P81">
-        <v>1.322646</v>
+        <v>1.0522130000000001</v>
       </c>
       <c r="X81" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="82" spans="1:24" x14ac:dyDescent="0.35">

</xml_diff>